<commit_message>
Conformist bias time averaging
</commit_message>
<xml_diff>
--- a/data/conf_snap_output/conf_snap_N.xlsx
+++ b/data/conf_snap_output/conf_snap_N.xlsx
@@ -362,7 +362,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>µ</t>
+          <t>mu</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -382,7 +382,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>α</t>
+          <t>alpha</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -425,17 +425,11 @@
       <c r="F2">
         <v>0.05</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
       <c r="I2">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -457,17 +451,11 @@
       <c r="F3">
         <v>0.05</v>
       </c>
-      <c r="G3">
-        <v>0.75</v>
-      </c>
-      <c r="H3">
-        <v>0.25</v>
-      </c>
       <c r="I3">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -489,17 +477,11 @@
       <c r="F4">
         <v>0.05</v>
       </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
       <c r="I4">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -528,10 +510,10 @@
         <v>1</v>
       </c>
       <c r="I5">
-        <v>0.96</v>
+        <v>0.8</v>
       </c>
       <c r="J5">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -560,10 +542,10 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="J6">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -595,7 +577,7 @@
         <v>0.9</v>
       </c>
       <c r="J7">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -624,10 +606,10 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="J8">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -656,10 +638,10 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>0.78</v>
+        <v>0.7</v>
       </c>
       <c r="J9">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -688,10 +670,10 @@
         <v>1</v>
       </c>
       <c r="I10">
-        <v>0.5600000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="J10">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -714,16 +696,16 @@
         <v>0.05</v>
       </c>
       <c r="G11">
-        <v>0.05128205128205128</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>0.9487179487179487</v>
+        <v>1</v>
       </c>
       <c r="I11">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="J11">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -746,16 +728,16 @@
         <v>0.05</v>
       </c>
       <c r="G12">
-        <v>0.02127659574468085</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>0.9787234042553191</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="J12">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -778,16 +760,16 @@
         <v>0.05</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I13">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -810,16 +792,16 @@
         <v>0.05</v>
       </c>
       <c r="G14">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="H14">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -842,16 +824,16 @@
         <v>0.05</v>
       </c>
       <c r="G15">
-        <v>0.06</v>
+        <v>0.2</v>
       </c>
       <c r="H15">
-        <v>0.9399999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="J15">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +856,16 @@
         <v>0.05</v>
       </c>
       <c r="G16">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conformist bias bug fix
</commit_message>
<xml_diff>
--- a/data/conf_snap_output/conf_snap_N.xlsx
+++ b/data/conf_snap_output/conf_snap_N.xlsx
@@ -425,11 +425,17 @@
       <c r="F2">
         <v>0.05</v>
       </c>
+      <c r="G2">
+        <v>0.2692307692307692</v>
+      </c>
+      <c r="H2">
+        <v>0.7307692307692307</v>
+      </c>
       <c r="I2">
-        <v>1</v>
+        <v>0.974</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
@@ -451,11 +457,17 @@
       <c r="F3">
         <v>0.05</v>
       </c>
+      <c r="G3">
+        <v>0.5</v>
+      </c>
+      <c r="H3">
+        <v>0.5</v>
+      </c>
       <c r="I3">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4">
@@ -477,11 +489,17 @@
       <c r="F4">
         <v>0.05</v>
       </c>
+      <c r="G4">
+        <v>0.09523809523809523</v>
+      </c>
+      <c r="H4">
+        <v>0.9047619047619048</v>
+      </c>
       <c r="I4">
-        <v>1</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="5">
@@ -504,16 +522,16 @@
         <v>0.05</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>0.119047619047619</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0.8809523809523809</v>
       </c>
       <c r="I5">
-        <v>0.8</v>
+        <v>0.958</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6">
@@ -542,10 +560,10 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>0.9</v>
+        <v>0.968</v>
       </c>
       <c r="J6">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -574,10 +592,10 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0.9</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="J7">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8">
@@ -606,10 +624,10 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.9</v>
+        <v>0.844</v>
       </c>
       <c r="J8">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9">
@@ -632,16 +650,16 @@
         <v>0.05</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>0.007142857142857143</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0.9928571428571429</v>
       </c>
       <c r="I9">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
@@ -664,16 +682,16 @@
         <v>0.05</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>0.006211180124223602</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0.9937888198757764</v>
       </c>
       <c r="I10">
-        <v>0.1</v>
+        <v>0.517</v>
       </c>
       <c r="J10">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11">
@@ -696,16 +714,16 @@
         <v>0.05</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>0.0163265306122449</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0.9836734693877551</v>
       </c>
       <c r="I11">
-        <v>0.1</v>
+        <v>0.265</v>
       </c>
       <c r="J11">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12">
@@ -728,16 +746,16 @@
         <v>0.05</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>0.04017857142857143</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0.9598214285714286</v>
       </c>
       <c r="I12">
-        <v>0.1</v>
+        <v>0.104</v>
       </c>
       <c r="J12">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13">
@@ -760,16 +778,16 @@
         <v>0.05</v>
       </c>
       <c r="G13">
-        <v>0.1</v>
+        <v>0.05268595041322314</v>
       </c>
       <c r="H13">
-        <v>0.9</v>
+        <v>0.9473140495867769</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="J13">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14">
@@ -792,16 +810,16 @@
         <v>0.05</v>
       </c>
       <c r="G14">
-        <v>0.1</v>
+        <v>0.1038696537678208</v>
       </c>
       <c r="H14">
-        <v>0.9</v>
+        <v>0.8961303462321792</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J14">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15">
@@ -824,16 +842,16 @@
         <v>0.05</v>
       </c>
       <c r="G15">
-        <v>0.2</v>
+        <v>0.1178247734138973</v>
       </c>
       <c r="H15">
-        <v>0.8</v>
+        <v>0.8821752265861027</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>0.007</v>
       </c>
       <c r="J15">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="16">
@@ -856,16 +874,16 @@
         <v>0.05</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>0.1461461461461462</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0.8538538538538538</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="J16">
-        <v>10</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polished version for publication
</commit_message>
<xml_diff>
--- a/data/conf_snap_output/conf_snap_N.xlsx
+++ b/data/conf_snap_output/conf_snap_N.xlsx
@@ -426,13 +426,13 @@
         <v>0.05</v>
       </c>
       <c r="G2">
-        <v>0.2692307692307692</v>
+        <v>0.3529411764705883</v>
       </c>
       <c r="H2">
-        <v>0.7307692307692307</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="I2">
-        <v>0.974</v>
+        <v>0.966</v>
       </c>
       <c r="J2">
         <v>1000</v>
@@ -458,13 +458,13 @@
         <v>0.05</v>
       </c>
       <c r="G3">
-        <v>0.5</v>
+        <v>0.3947368421052632</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>0.6052631578947368</v>
       </c>
       <c r="I3">
-        <v>0.958</v>
+        <v>0.962</v>
       </c>
       <c r="J3">
         <v>1000</v>
@@ -490,13 +490,13 @@
         <v>0.05</v>
       </c>
       <c r="G4">
-        <v>0.09523809523809523</v>
+        <v>0.06382978723404255</v>
       </c>
       <c r="H4">
-        <v>0.9047619047619048</v>
+        <v>0.9361702127659575</v>
       </c>
       <c r="I4">
-        <v>0.9370000000000001</v>
+        <v>0.953</v>
       </c>
       <c r="J4">
         <v>1000</v>
@@ -522,13 +522,13 @@
         <v>0.05</v>
       </c>
       <c r="G5">
-        <v>0.119047619047619</v>
+        <v>0.04166666666666666</v>
       </c>
       <c r="H5">
-        <v>0.8809523809523809</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="I5">
-        <v>0.958</v>
+        <v>0.952</v>
       </c>
       <c r="J5">
         <v>1000</v>
@@ -560,7 +560,7 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>0.968</v>
+        <v>0.949</v>
       </c>
       <c r="J6">
         <v>1000</v>
@@ -592,7 +592,7 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0.9350000000000001</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="J7">
         <v>1000</v>
@@ -624,7 +624,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.844</v>
+        <v>0.853</v>
       </c>
       <c r="J8">
         <v>1000</v>
@@ -650,13 +650,13 @@
         <v>0.05</v>
       </c>
       <c r="G9">
-        <v>0.007142857142857143</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0.9928571428571429</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>0.72</v>
+        <v>0.716</v>
       </c>
       <c r="J9">
         <v>1000</v>
@@ -682,13 +682,13 @@
         <v>0.05</v>
       </c>
       <c r="G10">
-        <v>0.006211180124223602</v>
+        <v>0.0130718954248366</v>
       </c>
       <c r="H10">
-        <v>0.9937888198757764</v>
+        <v>0.9869281045751634</v>
       </c>
       <c r="I10">
-        <v>0.517</v>
+        <v>0.541</v>
       </c>
       <c r="J10">
         <v>1000</v>
@@ -714,13 +714,13 @@
         <v>0.05</v>
       </c>
       <c r="G11">
-        <v>0.0163265306122449</v>
+        <v>0.0102827763496144</v>
       </c>
       <c r="H11">
-        <v>0.9836734693877551</v>
+        <v>0.9897172236503856</v>
       </c>
       <c r="I11">
-        <v>0.265</v>
+        <v>0.222</v>
       </c>
       <c r="J11">
         <v>1000</v>
@@ -746,13 +746,13 @@
         <v>0.05</v>
       </c>
       <c r="G12">
-        <v>0.04017857142857143</v>
+        <v>0.03651987110633727</v>
       </c>
       <c r="H12">
-        <v>0.9598214285714286</v>
+        <v>0.9634801288936627</v>
       </c>
       <c r="I12">
-        <v>0.104</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="J12">
         <v>1000</v>
@@ -778,13 +778,13 @@
         <v>0.05</v>
       </c>
       <c r="G13">
-        <v>0.05268595041322314</v>
+        <v>0.03516028955532575</v>
       </c>
       <c r="H13">
-        <v>0.9473140495867769</v>
+        <v>0.9648397104446742</v>
       </c>
       <c r="I13">
-        <v>0.032</v>
+        <v>0.033</v>
       </c>
       <c r="J13">
         <v>1000</v>
@@ -810,13 +810,13 @@
         <v>0.05</v>
       </c>
       <c r="G14">
-        <v>0.1038696537678208</v>
+        <v>0.09644670050761421</v>
       </c>
       <c r="H14">
-        <v>0.8961303462321792</v>
+        <v>0.9035532994923858</v>
       </c>
       <c r="I14">
-        <v>0.018</v>
+        <v>0.015</v>
       </c>
       <c r="J14">
         <v>1000</v>
@@ -842,13 +842,13 @@
         <v>0.05</v>
       </c>
       <c r="G15">
-        <v>0.1178247734138973</v>
+        <v>0.1362725450901804</v>
       </c>
       <c r="H15">
-        <v>0.8821752265861027</v>
+        <v>0.8637274549098196</v>
       </c>
       <c r="I15">
-        <v>0.007</v>
+        <v>0.002</v>
       </c>
       <c r="J15">
         <v>1000</v>
@@ -874,10 +874,10 @@
         <v>0.05</v>
       </c>
       <c r="G16">
-        <v>0.1461461461461462</v>
+        <v>0.1741741741741742</v>
       </c>
       <c r="H16">
-        <v>0.8538538538538538</v>
+        <v>0.8258258258258259</v>
       </c>
       <c r="I16">
         <v>0.001</v>

</xml_diff>